<commit_message>
Add rendered flow-diagram sheet to the Excel STTM output
Embeds a Graphviz-rendered boxes-and-arrows flowchart image as the first
sheet of the generated workbook, alongside the existing Table/Column
Lineage sheets, so the lineage can be seen at a glance rather than only
read as rows. Degrades gracefully (skips the sheet, adds a warning) if
Graphviz's `dot` executable isn't installed. Also fixes a real bug found
while wiring this up: node ids containing ":" (e.g. "table:foo.bar") were
being misinterpreted by Graphviz's DOT syntax as node:port references.
</commit_message>
<xml_diff>
--- a/input/sample_banking_dw_lineage_mapping.xlsx
+++ b/input/sample_banking_dw_lineage_mapping.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Lineage" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column Lineage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flow Diagram" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Lineage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column Lineage" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -136,6 +137,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7515225" cy="2209800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -452,6 +483,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -602,7 +647,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -855,7 +900,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>total_deposits_usd</t>
+          <t>total_withdrawals_usd</t>
         </is>
       </c>
     </row>
@@ -877,7 +922,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>total_withdrawals_usd</t>
+          <t>total_deposits_usd</t>
         </is>
       </c>
     </row>

</xml_diff>